<commit_message>
Complete Nifty100 Analytics Platform
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -500,7 +500,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>34.50618567955337</v>
+      </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="b">
         <v>0</v>
@@ -828,7 +830,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>15.56823256217168</v>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="b">
         <v>0</v>
@@ -910,7 +914,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>20.63103849143375</v>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="b">
         <v>0</v>
@@ -992,7 +998,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>27.2167818274256</v>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="b">
         <v>0</v>
@@ -1156,7 +1164,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>19.46310700548934</v>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="b">
         <v>0</v>
@@ -1238,7 +1248,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>37.29762744346468</v>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="b">
         <v>0</v>
@@ -1279,7 +1291,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>24.30118345247379</v>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="b">
         <v>0</v>
@@ -1320,7 +1334,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>21.81530931380111</v>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="b">
         <v>0</v>
@@ -1361,7 +1377,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>5.247691552181655</v>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="b">
         <v>0</v>
@@ -1484,7 +1502,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>5.863057152249307</v>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="b">
         <v>0</v>
@@ -1525,7 +1545,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>13.93946746062713</v>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="b">
         <v>0</v>
@@ -1566,7 +1588,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>14.43934874408408</v>
+      </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="b">
         <v>0</v>
@@ -1607,7 +1631,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>-11.76910917974342</v>
+      </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="b">
         <v>0</v>
@@ -1894,7 +1920,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>-5.002096841865733</v>
+      </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="b">
         <v>0</v>
@@ -1935,7 +1963,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>-3.469343496883137</v>
+      </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="b">
         <v>0</v>
@@ -1976,7 +2006,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="n">
+        <v>22.21293464748597</v>
+      </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="b">
         <v>0</v>
@@ -2099,7 +2131,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="n">
+        <v>8.674914145052593</v>
+      </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="b">
         <v>0</v>
@@ -2181,7 +2215,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
+      <c r="G43" t="n">
+        <v>9.689663003888427</v>
+      </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="b">
         <v>0</v>
@@ -2263,7 +2299,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="G45" t="n">
+        <v>32.49553261764786</v>
+      </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="b">
         <v>0</v>
@@ -2427,7 +2465,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="n">
+        <v>14.69779172398365</v>
+      </c>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="b">
         <v>0</v>
@@ -2468,7 +2508,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
+      <c r="G50" t="n">
+        <v>84.86188044662759</v>
+      </c>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="b">
         <v>0</v>
@@ -2509,7 +2551,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>45.37464474156747</v>
+      </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="b">
         <v>0</v>
@@ -2591,7 +2635,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
+      <c r="G53" t="n">
+        <v>17.36255738803865</v>
+      </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="b">
         <v>0</v>
@@ -2673,7 +2719,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="n">
+        <v>-19.25925925925925</v>
+      </c>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="b">
         <v>0</v>
@@ -2837,7 +2885,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
+      <c r="G59" t="n">
+        <v>-48.21728841371581</v>
+      </c>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="b">
         <v>0</v>
@@ -2960,7 +3010,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
+      <c r="G62" t="n">
+        <v>14.79620583960055</v>
+      </c>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="b">
         <v>0</v>
@@ -3042,7 +3094,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
+      <c r="G64" t="n">
+        <v>16.27250444793893</v>
+      </c>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="b">
         <v>0</v>
@@ -3083,7 +3137,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
+      <c r="G65" t="n">
+        <v>7.992990088177754</v>
+      </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="b">
         <v>0</v>
@@ -3165,7 +3221,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
+      <c r="G67" t="n">
+        <v>7.289119583372683</v>
+      </c>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="b">
         <v>0</v>
@@ -3206,7 +3264,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
+      <c r="G68" t="n">
+        <v>-3.978114349162654</v>
+      </c>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="b">
         <v>0</v>
@@ -3370,7 +3430,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
+      <c r="G72" t="n">
+        <v>10.20304470835676</v>
+      </c>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="b">
         <v>0</v>
@@ -3534,7 +3596,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
+      <c r="G76" t="n">
+        <v>15.44024389751422</v>
+      </c>
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="b">
         <v>0</v>
@@ -3616,7 +3680,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="n">
+        <v>-1.755412278125101</v>
+      </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="b">
         <v>0</v>
@@ -3657,7 +3723,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="G79" t="n">
+        <v>6.898030378675513</v>
+      </c>
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="b">
         <v>0</v>
@@ -3784,7 +3852,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
+      <c r="G82" t="n">
+        <v>24.94023133872936</v>
+      </c>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="b">
         <v>0</v>
@@ -3825,7 +3895,9 @@
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
+      <c r="G83" t="n">
+        <v>-16.81479293772952</v>
+      </c>
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="b">
         <v>0</v>
@@ -3948,7 +4020,9 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
+      <c r="G86" t="n">
+        <v>18.48596311592985</v>
+      </c>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="b">
         <v>0</v>
@@ -3989,7 +4063,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="n">
+        <v>22.16154572105831</v>
+      </c>
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="b">
         <v>0</v>
@@ -4030,7 +4106,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
+      <c r="G88" t="n">
+        <v>32.28517405641733</v>
+      </c>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="b">
         <v>0</v>
@@ -4071,7 +4149,9 @@
           <t>Asset Light</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
+      <c r="G89" t="n">
+        <v>12.53074535363581</v>
+      </c>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="b">
         <v>0</v>

</xml_diff>